<commit_message>
v1.20 Change 15: Seed updates for v1.20
- master_seed.xlsx updated: spawned Demand names have no Function suffix,
  created_under_function_id set on every Project, Project 5 (MBM Foundation
  Library) configured as DM-only, all activity_* column names in place
- seed.json regenerated from workbook (6 Projects, 11 Demands, 18 People)
- REQUIREMENTS.md updated to v1.20 full spec
- DESIGN.md renamed to DESIGNSYSTEM.md (spec section 7 reference updated)
- docs/CAPACITY_AUDIT.md removed (superseded by seed reconciliation table in spec)
- Stray empty files and one-time patch script cleaned up

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/seed/master_seed.xlsx
+++ b/seed/master_seed.xlsx
@@ -65,7 +65,7 @@
     <t>Sarah Chen</t>
   </si>
   <si>
-    <t>Feasibility study for Plant D MES infrastructure upgrade. Draft â€” requirements not yet defined.</t>
+    <t>Feasibility study for Plant D MES infrastructure upgrade. Draft ”” requirements not yet defined.</t>
   </si>
   <si>
     <t>Digital Manufacturing, Group IT Enterprise Solutions</t>
@@ -101,7 +101,7 @@
     <t>Anya Petrov</t>
   </si>
   <si>
-    <t>Enterprise data lake build. Cross-Function: DM MI&amp;V + GroupIT Data &amp; Integration. No Programme â€” demonstrates Unaligned Projects card.</t>
+    <t>Enterprise data lake build. Cross-Function: DM MI&amp;V + GroupIT Data &amp; Integration. No Programme ”” demonstrates Unaligned Projects card.</t>
   </si>
   <si>
     <t>Submitted</t>
@@ -230,7 +230,7 @@
     <t>Migration Support</t>
   </si>
   <si>
-    <t>direct:MES Super User support â€” Plant B</t>
+    <t>direct:MES Super User support ”” Plant B</t>
   </si>
   <si>
     <t>Ongoing support</t>
@@ -302,7 +302,7 @@
     <t>Integration Architecture</t>
   </si>
   <si>
-    <t>Spawn-time value 60h/mo â€” DM Demand drifted to 80h post-spawn</t>
+    <t>Spawn-time value 60h/mo ”” DM Demand drifted to 80h post-spawn</t>
   </si>
   <si>
     <t>Production Workflow Design</t>
@@ -494,13 +494,13 @@
     <t>function_name</t>
   </si>
   <si>
-    <t>Manufacturing Operations Management â€” MES, order execution, production tracking, OEE.</t>
-  </si>
-  <si>
-    <t>Manufacturing Intelligence &amp; Visualisation â€” historians, analytics, dashboards, reporting.</t>
-  </si>
-  <si>
-    <t>Model-Based Manufacturing â€” simulation, digital twins, process modelling.</t>
+    <t>Manufacturing Operations Management ”” MES, order execution, production tracking, OEE.</t>
+  </si>
+  <si>
+    <t>Manufacturing Intelligence &amp; Visualisation ”” historians, analytics, dashboards, reporting.</t>
+  </si>
+  <si>
+    <t>Model-Based Manufacturing ”” simulation, digital twins, process modelling.</t>
   </si>
   <si>
     <t>Cloud infrastructure, network engineering, and platform services for the enterprise.</t>
@@ -593,7 +593,7 @@
     <t>Yuki Watanabe</t>
   </si>
   <si>
-    <t>Henrik SÃ¸rensen</t>
+    <t>Henrik Sørensen</t>
   </si>
   <si>
     <t>person_name</t>
@@ -632,19 +632,19 @@
     <t>Ad-hoc shift pattern review</t>
   </si>
   <si>
-    <t>Ad-hoc review of MES shift patterns at Plant A. 1 phase, 1 MOM Basic requirement. No external.</t>
+    <t>Ad-hoc review of MES shift patterns at Plant A. 1 Activity, 1 MOM Basic requirement. No external.</t>
   </si>
   <si>
     <t>Plant A SCADA migration assist</t>
   </si>
   <si>
-    <t>Assist with SCADA migration at Plant A. Submitted â€” Approve is the next-step CTA.</t>
-  </si>
-  <si>
-    <t>MES Super User support â€” Plant B</t>
-  </si>
-  <si>
-    <t>Ongoing BAU MES super user support at Plant B. Indefinite phase; partial allocation in place. Has Other Internal Team external requirement.</t>
+    <t>Assist with SCADA migration at Plant A. Submitted ”” Approve is the next-step CTA.</t>
+  </si>
+  <si>
+    <t>MES Super User support ”” Plant B</t>
+  </si>
+  <si>
+    <t>Ongoing BAU MES super user support at Plant B. Indefinite Activity; partial allocation in place. Has Other Internal Team external requirement.</t>
   </si>
   <si>
     <t>PartiallyAllocated</t>
@@ -665,7 +665,7 @@
     <t>demand_name</t>
   </si>
   <si>
-    <t>Partial â€” 20 hrs/mo unplanned</t>
+    <t>Partial ”” 20 hrs/mo unplanned</t>
   </si>
 </sst>
 </file>
@@ -1225,7 +1225,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1274,7 +1274,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1367,7 +1367,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1647,7 +1647,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1747,7 +1747,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2146,7 +2146,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2980,7 +2980,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3082,7 +3082,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3142,7 +3142,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3191,7 +3191,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3330,7 +3330,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3649,7 +3649,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3921,7 +3921,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4696,7 +4696,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4853,7 +4853,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4900,7 +4900,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5180,7 +5180,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5229,7 +5229,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5268,7 +5268,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5315,6 +5315,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>